<commit_message>
Full pipeline updates after changing joint approximation
</commit_message>
<xml_diff>
--- a/Figures/tab_MOIs_edited.xlsx
+++ b/Figures/tab_MOIs_edited.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ataylor/Documents/PvMolCorrection/Figures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1269D2F1-BA22-9645-B416-59E6389CABF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36E25915-4A50-E742-92AF-AB1D1055005F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25520" yWindow="500" windowWidth="38400" windowHeight="19860" xr2:uid="{C38C7C08-B65B-444B-A243-889EF7BF4B18}"/>
+    <workbookView xWindow="34560" yWindow="600" windowWidth="38400" windowHeight="19200" xr2:uid="{C38C7C08-B65B-444B-A243-889EF7BF4B18}"/>
   </bookViews>
   <sheets>
     <sheet name="tab_MOIs_edited" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">tab_MOIs_edited!$A$1:$V$59</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -97,18 +100,12 @@
     <t>AS</t>
   </si>
   <si>
-    <t>CHQ/PMQ</t>
-  </si>
-  <si>
     <t>VHX_583</t>
   </si>
   <si>
     <t>VHX_203</t>
   </si>
   <si>
-    <t>CHQ</t>
-  </si>
-  <si>
     <t>VHX_400</t>
   </si>
   <si>
@@ -269,6 +266,12 @@
   </si>
   <si>
     <t>VHX_646</t>
+  </si>
+  <si>
+    <t>CQ/PQ</t>
+  </si>
+  <si>
+    <t>CQ</t>
   </si>
 </sst>
 </file>
@@ -1202,6 +1205,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65B06858-4ADD-8748-A4B4-48F3DA5B81DB}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:V59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1368,7 +1374,7 @@
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B4" s="1">
         <v>4</v>
@@ -1422,7 +1428,7 @@
         <v>3</v>
       </c>
       <c r="S4" s="1" t="s">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="T4" s="8"/>
       <c r="U4" s="4"/>
@@ -1430,7 +1436,7 @@
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B5" s="1">
         <v>1</v>
@@ -1484,7 +1490,7 @@
         <v>4</v>
       </c>
       <c r="S5" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T5" s="9"/>
       <c r="U5" s="9"/>
@@ -1492,7 +1498,7 @@
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B6" s="1">
         <v>1</v>
@@ -1546,7 +1552,7 @@
         <v>4</v>
       </c>
       <c r="S6" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T6" s="9"/>
       <c r="U6" s="9"/>
@@ -1554,7 +1560,7 @@
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B7" s="1">
         <v>1</v>
@@ -1608,7 +1614,7 @@
         <v>4</v>
       </c>
       <c r="S7" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T7" s="9"/>
       <c r="U7" s="9"/>
@@ -1616,7 +1622,7 @@
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B8" s="1">
         <v>2</v>
@@ -1670,7 +1676,7 @@
         <v>4</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T8" s="9"/>
       <c r="U8" s="9"/>
@@ -1678,7 +1684,7 @@
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B9" s="1">
         <v>1</v>
@@ -1732,7 +1738,7 @@
         <v>4</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T9" s="9"/>
       <c r="U9" s="9"/>
@@ -1740,7 +1746,7 @@
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B10" s="1">
         <v>2</v>
@@ -1794,7 +1800,7 @@
         <v>4</v>
       </c>
       <c r="S10" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T10" s="9"/>
       <c r="U10" s="9"/>
@@ -1802,7 +1808,7 @@
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B11" s="1">
         <v>2</v>
@@ -1856,7 +1862,7 @@
         <v>4</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T11" s="9"/>
       <c r="U11" s="9"/>
@@ -1864,7 +1870,7 @@
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B12" s="1">
         <v>3</v>
@@ -1918,7 +1924,7 @@
         <v>4</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T12" s="9"/>
       <c r="U12" s="9"/>
@@ -1926,7 +1932,7 @@
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B13" s="1">
         <v>3</v>
@@ -1980,7 +1986,7 @@
         <v>5</v>
       </c>
       <c r="S13" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T13" s="10"/>
       <c r="U13" s="10"/>
@@ -1988,7 +1994,7 @@
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B14" s="1">
         <v>1</v>
@@ -2042,7 +2048,7 @@
         <v>5</v>
       </c>
       <c r="S14" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T14" s="9"/>
       <c r="U14" s="9"/>
@@ -2050,7 +2056,7 @@
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B15" s="1">
         <v>1</v>
@@ -2104,7 +2110,7 @@
         <v>5</v>
       </c>
       <c r="S15" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T15" s="9"/>
       <c r="U15" s="9"/>
@@ -2112,7 +2118,7 @@
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B16" s="1">
         <v>1</v>
@@ -2166,7 +2172,7 @@
         <v>5</v>
       </c>
       <c r="S16" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T16" s="9"/>
       <c r="U16" s="9"/>
@@ -2174,7 +2180,7 @@
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B17" s="1">
         <v>1</v>
@@ -2228,7 +2234,7 @@
         <v>5</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T17" s="9"/>
       <c r="U17" s="9"/>
@@ -2236,7 +2242,7 @@
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B18" s="1">
         <v>2</v>
@@ -2290,7 +2296,7 @@
         <v>5</v>
       </c>
       <c r="S18" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T18" s="9"/>
       <c r="U18" s="9"/>
@@ -2298,7 +2304,7 @@
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B19" s="1">
         <v>2</v>
@@ -2352,7 +2358,7 @@
         <v>5</v>
       </c>
       <c r="S19" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T19" s="9"/>
       <c r="U19" s="9"/>
@@ -2360,7 +2366,7 @@
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B20" s="1">
         <v>3</v>
@@ -2414,7 +2420,7 @@
         <v>5</v>
       </c>
       <c r="S20" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T20" s="9"/>
       <c r="U20" s="9"/>
@@ -2422,7 +2428,7 @@
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B21" s="1">
         <v>2</v>
@@ -2476,7 +2482,7 @@
         <v>5</v>
       </c>
       <c r="S21" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T21" s="9"/>
       <c r="U21" s="9"/>
@@ -2484,7 +2490,7 @@
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B22" s="1">
         <v>3</v>
@@ -2538,7 +2544,7 @@
         <v>5</v>
       </c>
       <c r="S22" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T22" s="9"/>
       <c r="U22" s="9"/>
@@ -2546,7 +2552,7 @@
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B23" s="1">
         <v>1</v>
@@ -2600,7 +2606,7 @@
         <v>6</v>
       </c>
       <c r="S23" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T23" s="9"/>
       <c r="U23" s="9"/>
@@ -2608,7 +2614,7 @@
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B24" s="1">
         <v>1</v>
@@ -2662,7 +2668,7 @@
         <v>6</v>
       </c>
       <c r="S24" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T24" s="9"/>
       <c r="U24" s="9"/>
@@ -2670,7 +2676,7 @@
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B25" s="1">
         <v>1</v>
@@ -2724,7 +2730,7 @@
         <v>6</v>
       </c>
       <c r="S25" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T25" s="9"/>
       <c r="U25" s="9"/>
@@ -2732,7 +2738,7 @@
     </row>
     <row r="26" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B26" s="1">
         <v>2</v>
@@ -2786,7 +2792,7 @@
         <v>6</v>
       </c>
       <c r="S26" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T26" s="9"/>
       <c r="U26" s="9"/>
@@ -2794,7 +2800,7 @@
     </row>
     <row r="27" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B27" s="1">
         <v>2</v>
@@ -2848,7 +2854,7 @@
         <v>6</v>
       </c>
       <c r="S27" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T27" s="9"/>
       <c r="U27" s="9"/>
@@ -2856,7 +2862,7 @@
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B28" s="1">
         <v>2</v>
@@ -2910,7 +2916,7 @@
         <v>6</v>
       </c>
       <c r="S28" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T28" s="9"/>
       <c r="U28" s="9"/>
@@ -2918,7 +2924,7 @@
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B29" s="1">
         <v>2</v>
@@ -2972,7 +2978,7 @@
         <v>6</v>
       </c>
       <c r="S29" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T29" s="9"/>
       <c r="U29" s="9"/>
@@ -2980,7 +2986,7 @@
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B30" s="1">
         <v>3</v>
@@ -3034,7 +3040,7 @@
         <v>7</v>
       </c>
       <c r="S30" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T30" s="10"/>
       <c r="U30" s="10"/>
@@ -3042,7 +3048,7 @@
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B31" s="1">
         <v>2</v>
@@ -3096,7 +3102,7 @@
         <v>7</v>
       </c>
       <c r="S31" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T31" s="9"/>
       <c r="U31" s="9"/>
@@ -3104,7 +3110,7 @@
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B32" s="1">
         <v>1</v>
@@ -3158,7 +3164,7 @@
         <v>7</v>
       </c>
       <c r="S32" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T32" s="9"/>
       <c r="U32" s="9"/>
@@ -3166,7 +3172,7 @@
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B33" s="1">
         <v>1</v>
@@ -3220,7 +3226,7 @@
         <v>7</v>
       </c>
       <c r="S33" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T33" s="9"/>
       <c r="U33" s="9"/>
@@ -3228,7 +3234,7 @@
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B34" s="1">
         <v>1</v>
@@ -3282,7 +3288,7 @@
         <v>7</v>
       </c>
       <c r="S34" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T34" s="9"/>
       <c r="U34" s="9"/>
@@ -3290,7 +3296,7 @@
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B35" s="1">
         <v>1</v>
@@ -3344,7 +3350,7 @@
         <v>7</v>
       </c>
       <c r="S35" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T35" s="9"/>
       <c r="U35" s="9"/>
@@ -3352,7 +3358,7 @@
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B36" s="1">
         <v>1</v>
@@ -3406,7 +3412,7 @@
         <v>8</v>
       </c>
       <c r="S36" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T36" s="9"/>
       <c r="U36" s="9"/>
@@ -3414,7 +3420,7 @@
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B37" s="1">
         <v>2</v>
@@ -3468,7 +3474,7 @@
         <v>8</v>
       </c>
       <c r="S37" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T37" s="9"/>
       <c r="U37" s="9"/>
@@ -3476,7 +3482,7 @@
     </row>
     <row r="38" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B38" s="1">
         <v>1</v>
@@ -3530,7 +3536,7 @@
         <v>8</v>
       </c>
       <c r="S38" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T38" s="9"/>
       <c r="U38" s="9"/>
@@ -3538,7 +3544,7 @@
     </row>
     <row r="39" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B39" s="1">
         <v>1</v>
@@ -3592,7 +3598,7 @@
         <v>8</v>
       </c>
       <c r="S39" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T39" s="9"/>
       <c r="U39" s="9"/>
@@ -3600,7 +3606,7 @@
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B40" s="1">
         <v>1</v>
@@ -3654,7 +3660,7 @@
         <v>8</v>
       </c>
       <c r="S40" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T40" s="9"/>
       <c r="U40" s="9"/>
@@ -3662,7 +3668,7 @@
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B41" s="1">
         <v>1</v>
@@ -3716,7 +3722,7 @@
         <v>8</v>
       </c>
       <c r="S41" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T41" s="9"/>
       <c r="U41" s="9"/>
@@ -3724,7 +3730,7 @@
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B42" s="1">
         <v>2</v>
@@ -3778,7 +3784,7 @@
         <v>8</v>
       </c>
       <c r="S42" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T42" s="9"/>
       <c r="U42" s="9"/>
@@ -3786,7 +3792,7 @@
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B43" s="1">
         <v>1</v>
@@ -3840,7 +3846,7 @@
         <v>8</v>
       </c>
       <c r="S43" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T43" s="9"/>
       <c r="U43" s="9"/>
@@ -3848,7 +3854,7 @@
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B44" s="1">
         <v>3</v>
@@ -3902,7 +3908,7 @@
         <v>8</v>
       </c>
       <c r="S44" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T44" s="9"/>
       <c r="U44" s="9"/>
@@ -3910,7 +3916,7 @@
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B45" s="1">
         <v>3</v>
@@ -3964,7 +3970,7 @@
         <v>8</v>
       </c>
       <c r="S45" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T45" s="9"/>
       <c r="U45" s="9"/>
@@ -3972,7 +3978,7 @@
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B46" s="1">
         <v>3</v>
@@ -4034,7 +4040,7 @@
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B47" s="1">
         <v>1</v>
@@ -4088,7 +4094,7 @@
         <v>9</v>
       </c>
       <c r="S47" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T47" s="9"/>
       <c r="U47" s="9"/>
@@ -4096,7 +4102,7 @@
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B48" s="1">
         <v>1</v>
@@ -4150,7 +4156,7 @@
         <v>9</v>
       </c>
       <c r="S48" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T48" s="9"/>
       <c r="U48" s="9"/>
@@ -4158,7 +4164,7 @@
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B49" s="1">
         <v>2</v>
@@ -4212,7 +4218,7 @@
         <v>9</v>
       </c>
       <c r="S49" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T49" s="9"/>
       <c r="U49" s="9"/>
@@ -4220,7 +4226,7 @@
     </row>
     <row r="50" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B50" s="1">
         <v>2</v>
@@ -4274,7 +4280,7 @@
         <v>9</v>
       </c>
       <c r="S50" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T50" s="9"/>
       <c r="U50" s="9"/>
@@ -4282,7 +4288,7 @@
     </row>
     <row r="51" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B51" s="1">
         <v>2</v>
@@ -4336,7 +4342,7 @@
         <v>9</v>
       </c>
       <c r="S51" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T51" s="9"/>
       <c r="U51" s="9"/>
@@ -4344,7 +4350,7 @@
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B52" s="1">
         <v>3</v>
@@ -4398,7 +4404,7 @@
         <v>9</v>
       </c>
       <c r="S52" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T52" s="8"/>
       <c r="U52" s="4"/>
@@ -4406,7 +4412,7 @@
     </row>
     <row r="53" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B53" s="1">
         <v>1</v>
@@ -4460,7 +4466,7 @@
         <v>10</v>
       </c>
       <c r="S53" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T53" s="9"/>
       <c r="U53" s="9"/>
@@ -4468,7 +4474,7 @@
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B54" s="1">
         <v>1</v>
@@ -4522,7 +4528,7 @@
         <v>10</v>
       </c>
       <c r="S54" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T54" s="9"/>
       <c r="U54" s="9"/>
@@ -4530,7 +4536,7 @@
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B55" s="1">
         <v>1</v>
@@ -4584,7 +4590,7 @@
         <v>10</v>
       </c>
       <c r="S55" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T55" s="9"/>
       <c r="U55" s="9"/>
@@ -4592,7 +4598,7 @@
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B56" s="1">
         <v>1</v>
@@ -4646,7 +4652,7 @@
         <v>10</v>
       </c>
       <c r="S56" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T56" s="9"/>
       <c r="U56" s="9"/>
@@ -4654,7 +4660,7 @@
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B57" s="1">
         <v>2</v>
@@ -4708,7 +4714,7 @@
         <v>10</v>
       </c>
       <c r="S57" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T57" s="9"/>
       <c r="U57" s="9"/>
@@ -4716,7 +4722,7 @@
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B58" s="1">
         <v>2</v>
@@ -4770,7 +4776,7 @@
         <v>11</v>
       </c>
       <c r="S58" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T58" s="9"/>
       <c r="U58" s="9"/>
@@ -4778,7 +4784,7 @@
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B59" s="1">
         <v>3</v>
@@ -4832,7 +4838,7 @@
         <v>14</v>
       </c>
       <c r="S59" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="T59" s="9"/>
       <c r="U59" s="9"/>
@@ -4903,7 +4909,8 @@
     <mergeCell ref="T55:U55"/>
     <mergeCell ref="T56:U56"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="53" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>